<commit_message>
Add DB helpers and refactor OrangeHRM flows
Introduce centralized DB utilities and refactor test flows for OrangeHRM. Added DBConnInfo, DBQueryExecutorHelper and OrangeHRMDBInfo to standardize DB connection and query execution; added database rule classes (CreateNewEmployeeDB, CreateNewUsernameDB, GetEmployeeDetailsDB, GetEmployeeLoginDetailsDB) and removed legacy EmployeeTable/UsernameTable. Moved model classes into apps.orangeHRM.models.*, relocated flow classes into rules packages and updated imports/usages. Enhanced page objects (LoginPage, AddEmployeePage) with account-disabled checks and success message assertion. Updated E2ETest to use new rules and DB helpers, added a disabled-user test path, and improved assertions. Also added a VSCode tasks.json, adjusted GlobalTestRunConfig (HEADLESS true, SLOWMOTION 200), and updated test suite tags. Includes a binary QA plan spreadsheet change.
</commit_message>
<xml_diff>
--- a/QAPlan_OrangeHRM-PIM_.xlsx
+++ b/QAPlan_OrangeHRM-PIM_.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\Repositorys\Playwright\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F21AFE-2F29-4389-80FB-E4C7C9E548A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B4CAFC-DB77-49E1-8EA1-EA3080D9B163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="877" firstSheet="6" activeTab="6" xr2:uid="{FD97303A-53B3-48AB-ABDA-C3D67ED6805C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="877" firstSheet="6" activeTab="7" xr2:uid="{FD97303A-53B3-48AB-ABDA-C3D67ED6805C}"/>
   </bookViews>
   <sheets>
     <sheet name="Version" sheetId="1" r:id="rId1"/>
@@ -1911,6 +1911,18 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1961,18 +1973,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4365,28 +4365,28 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="102" t="s">
+      <c r="B2" s="106" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="103"/>
-      <c r="D2" s="103"/>
-      <c r="E2" s="104"/>
+      <c r="C2" s="107"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="108"/>
     </row>
     <row r="3" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="105"/>
-      <c r="C3" s="106"/>
-      <c r="D3" s="106"/>
-      <c r="E3" s="107"/>
+      <c r="B3" s="109"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="111"/>
     </row>
     <row r="4" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="C4" s="108">
+      <c r="C4" s="112">
         <v>46022</v>
       </c>
-      <c r="D4" s="109"/>
-      <c r="E4" s="110"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="114"/>
     </row>
     <row r="5" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="28" t="s">
@@ -4447,85 +4447,85 @@
       <c r="E11" s="38"/>
     </row>
     <row r="12" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="111" t="s">
+      <c r="B12" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="112"/>
-      <c r="D12" s="112"/>
-      <c r="E12" s="113"/>
+      <c r="C12" s="116"/>
+      <c r="D12" s="116"/>
+      <c r="E12" s="117"/>
     </row>
     <row r="13" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="114" t="s">
+      <c r="C13" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="D13" s="114"/>
-      <c r="E13" s="115"/>
+      <c r="D13" s="118"/>
+      <c r="E13" s="119"/>
     </row>
     <row r="14" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="22">
         <v>1</v>
       </c>
-      <c r="C14" s="116" t="s">
+      <c r="C14" s="120" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="117"/>
-      <c r="E14" s="118"/>
+      <c r="D14" s="121"/>
+      <c r="E14" s="122"/>
     </row>
     <row r="15" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="22">
         <v>2</v>
       </c>
-      <c r="C15" s="119"/>
-      <c r="D15" s="119"/>
-      <c r="E15" s="120"/>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="103"/>
     </row>
     <row r="16" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="22">
         <v>3</v>
       </c>
-      <c r="C16" s="119"/>
-      <c r="D16" s="119"/>
-      <c r="E16" s="120"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="103"/>
     </row>
     <row r="17" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="22">
         <v>4</v>
       </c>
-      <c r="C17" s="119"/>
-      <c r="D17" s="119"/>
-      <c r="E17" s="120"/>
+      <c r="C17" s="102"/>
+      <c r="D17" s="102"/>
+      <c r="E17" s="103"/>
     </row>
     <row r="18" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="22">
         <v>5</v>
       </c>
-      <c r="C18" s="119"/>
-      <c r="D18" s="119"/>
-      <c r="E18" s="120"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="103"/>
     </row>
     <row r="19" spans="2:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="23">
         <v>6</v>
       </c>
-      <c r="C19" s="121"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="122"/>
+      <c r="C19" s="104"/>
+      <c r="D19" s="104"/>
+      <c r="E19" s="105"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B2:E3"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C14:E14"/>
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="C19:E19"/>
-    <mergeCell ref="B2:E3"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C14:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -6794,7 +6794,7 @@
         <v>72</v>
       </c>
       <c r="E2" s="51" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F2" s="50" t="s">
         <v>17</v>

</xml_diff>